<commit_message>
feat: final file for production with panel adjustment
</commit_message>
<xml_diff>
--- a/pcb/production/bom-list_sound.xlsx
+++ b/pcb/production/bom-list_sound.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\PROJECT\FBZCORP\pribadi\fastwork\NULL BADGE CITY\null-city-badge2 - Copy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\PROJECT\FBZCORP\pribadi\fastwork\NULL BADGE CITY\null-city-badge2 - Copy\production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E77C407-08F2-47CD-8E26-B1498E52B578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA0CABB-D72F-4C5E-B425-AD9A139B5400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bom" sheetId="1" r:id="rId1"/>
@@ -74,9 +74,6 @@
     <t>CL05A106MQ5NUNC</t>
   </si>
   <si>
-    <t>C29</t>
-  </si>
-  <si>
     <t>22U</t>
   </si>
   <si>
@@ -174,6 +171,9 @@
   </si>
   <si>
     <t>PZ254V-11-07P</t>
+  </si>
+  <si>
+    <t>C29, C31</t>
   </si>
 </sst>
 </file>
@@ -748,7 +748,7 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>7</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>7</v>
@@ -788,70 +788,70 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" t="s">
         <v>15</v>
-      </c>
-      <c r="G4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" t="s">
         <v>45</v>
       </c>
-      <c r="F5" t="s">
-        <v>46</v>
-      </c>
       <c r="G5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>7</v>
@@ -860,64 +860,64 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" t="s">
         <v>21</v>
       </c>
-      <c r="F7" t="s">
-        <v>22</v>
-      </c>
       <c r="G7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
         <v>24</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>25</v>
-      </c>
-      <c r="G8" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
         <v>27</v>
-      </c>
-      <c r="B9" t="s">
-        <v>28</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" t="s">
         <v>29</v>
-      </c>
-      <c r="F9" t="s">
-        <v>29</v>
-      </c>
-      <c r="G9" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F10">
         <v>1609</v>
@@ -925,15 +925,15 @@
     </row>
     <row r="13" spans="1:9">
       <c r="B13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s">
         <v>31</v>
-      </c>
-      <c r="D13" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="B14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>